<commit_message>
Capítulo 3: aplicación de la metodología al caso simulado
- Fases 0-4 sobre admisión y matrícula de la IES-S: madurez, RAT,
  dictamen de gran escala, 13 escenarios, riesgo inherente y residual,
  mapas de calor, EIPD de SP3, plan de tratamiento e indicadores.
- Pruebas de la plantilla (T-01 a T-06), verificación de requisitos,
  resultados, cronograma y presupuesto referencial.
- Matriz aplicada generada desde escenarios_IES-S.json; validación con
  expertos marcada como pendiente.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/matriz/Plantilla_Matriz_Riesgos_LOPDP.xlsx
+++ b/matriz/Plantilla_Matriz_Riesgos_LOPDP.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="377">
   <si>
     <t>Plantilla de matriz de riesgos del tratamiento de datos personales (LOPDP)</t>
   </si>
@@ -803,6 +803,33 @@
   </si>
   <si>
     <t>Autenticación multifactor para personal con acceso a datos de aspirantes</t>
+  </si>
+  <si>
+    <t>8.6</t>
+  </si>
+  <si>
+    <t>Gestión de la capacidad</t>
+  </si>
+  <si>
+    <t>Dimensionar el portal para los cierres de postulación</t>
+  </si>
+  <si>
+    <t>8.7</t>
+  </si>
+  <si>
+    <t>Protección contra malware</t>
+  </si>
+  <si>
+    <t>Protección de puestos de trabajo y servidores del proceso</t>
+  </si>
+  <si>
+    <t>8.8</t>
+  </si>
+  <si>
+    <t>Gestión de vulnerabilidades técnicas</t>
+  </si>
+  <si>
+    <t>Parcheo del SGA, portal y servidores en plazos definidos</t>
   </si>
   <si>
     <t>8.10</t>
@@ -1939,16 +1966,16 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>344</v>
+        <v>353</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>345</v>
+        <v>354</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>40</v>
@@ -1960,13 +1987,13 @@
         <v>60</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>347</v>
+        <v>356</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>348</v>
+        <v>357</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -1983,7 +2010,7 @@
         <v>16</v>
       </c>
       <c r="E2" s="37" t="s">
-        <v>349</v>
+        <v>358</v>
       </c>
       <c r="F2" s="37" t="s">
         <v>78</v>
@@ -1995,7 +2022,7 @@
         <v>0</v>
       </c>
       <c r="I2" s="37" t="s">
-        <v>350</v>
+        <v>359</v>
       </c>
       <c r="J2" s="37" t="s">
         <v>89</v>
@@ -2009,25 +2036,25 @@
         <v>90</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>351</v>
+        <v>360</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>352</v>
+        <v>361</v>
       </c>
       <c r="E3" s="37" t="s">
         <v>71</v>
       </c>
       <c r="F3" s="37" t="s">
-        <v>353</v>
+        <v>362</v>
       </c>
       <c r="G3" s="37" t="s">
-        <v>354</v>
+        <v>363</v>
       </c>
       <c r="H3" s="37">
         <v>1</v>
       </c>
       <c r="I3" s="37" t="s">
-        <v>355</v>
+        <v>364</v>
       </c>
       <c r="J3" s="37" t="s">
         <v>90</v>
@@ -2042,16 +2069,16 @@
       </c>
       <c r="C4" s="29"/>
       <c r="D4" s="37" t="s">
-        <v>356</v>
+        <v>365</v>
       </c>
       <c r="E4" s="37" t="s">
-        <v>357</v>
+        <v>366</v>
       </c>
       <c r="F4" s="37" t="s">
-        <v>358</v>
+        <v>367</v>
       </c>
       <c r="G4" s="37" t="s">
-        <v>359</v>
+        <v>368</v>
       </c>
       <c r="H4" s="37">
         <v>2</v>
@@ -2075,19 +2102,19 @@
         <v>192</v>
       </c>
       <c r="E5" s="37" t="s">
-        <v>360</v>
+        <v>369</v>
       </c>
       <c r="F5" s="37" t="s">
-        <v>361</v>
+        <v>370</v>
       </c>
       <c r="G5" s="37" t="s">
-        <v>362</v>
+        <v>371</v>
       </c>
       <c r="H5" s="37">
         <v>3</v>
       </c>
       <c r="I5" s="37" t="s">
-        <v>363</v>
+        <v>372</v>
       </c>
       <c r="J5" s="37" t="s">
         <v>76</v>
@@ -2105,11 +2132,11 @@
       <c r="E6" s="29"/>
       <c r="F6" s="29"/>
       <c r="G6" s="37" t="s">
-        <v>364</v>
+        <v>373</v>
       </c>
       <c r="H6" s="29"/>
       <c r="I6" s="37" t="s">
-        <v>365</v>
+        <v>374</v>
       </c>
       <c r="J6" s="37" t="s">
         <v>91</v>
@@ -2125,12 +2152,12 @@
       <c r="G7" s="29"/>
       <c r="H7" s="29"/>
       <c r="I7" s="37" t="s">
-        <v>366</v>
+        <v>375</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
     </row>
   </sheetData>
@@ -8498,7 +8525,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -8781,6 +8808,48 @@
       </c>
       <c r="D22" s="18" t="s">
         <v>277</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="18" t="s">
+        <v>278</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>279</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>282</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="D25" s="18" t="s">
+        <v>286</v>
       </c>
     </row>
   </sheetData>
@@ -8805,62 +8874,62 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>278</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>279</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>280</v>
+        <v>289</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>281</v>
+        <v>290</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>285</v>
+        <v>294</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>288</v>
+        <v>297</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -8868,7 +8937,7 @@
         <v>61</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="C5" s="23">
         <v>1</v>
@@ -11401,7 +11470,7 @@
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
     </row>
   </sheetData>
@@ -11447,12 +11516,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -11460,36 +11529,36 @@
         <v>28</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>300</v>
+        <v>309</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>285</v>
+        <v>294</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>304</v>
+        <v>313</v>
       </c>
       <c r="C5" s="26">
         <v>0.9</v>
@@ -11502,15 +11571,15 @@
         <v>1</v>
       </c>
       <c r="I5" s="28" t="s">
-        <v>305</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
-        <v>306</v>
+        <v>315</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>307</v>
+        <v>316</v>
       </c>
       <c r="C6" s="26">
         <v>0.7</v>
@@ -11523,15 +11592,15 @@
         <v>1</v>
       </c>
       <c r="I6" s="28" t="s">
-        <v>308</v>
+        <v>317</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
-        <v>309</v>
+        <v>318</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>310</v>
+        <v>319</v>
       </c>
       <c r="C7" s="26">
         <v>0.4</v>
@@ -11544,15 +11613,15 @@
         <v>0</v>
       </c>
       <c r="I7" s="28" t="s">
-        <v>311</v>
+        <v>320</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>312</v>
+        <v>321</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>313</v>
+        <v>322</v>
       </c>
       <c r="C8" s="26">
         <v>0.6</v>
@@ -11565,15 +11634,15 @@
         <v>1</v>
       </c>
       <c r="I8" s="28" t="s">
-        <v>314</v>
+        <v>323</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
-        <v>315</v>
+        <v>324</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="C9" s="26">
         <v>0.8</v>
@@ -11586,15 +11655,15 @@
         <v>1</v>
       </c>
       <c r="I9" s="28" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
       <c r="C10" s="26">
         <v>0.6</v>
@@ -11607,15 +11676,15 @@
         <v>1</v>
       </c>
       <c r="I10" s="28" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="C11" s="26">
         <v>0.3</v>
@@ -11628,15 +11697,15 @@
         <v>0</v>
       </c>
       <c r="I11" s="28" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
-        <v>324</v>
+        <v>333</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="C12" s="26">
         <v>0.9</v>
@@ -11649,15 +11718,15 @@
         <v>1</v>
       </c>
       <c r="I12" s="28" t="s">
-        <v>326</v>
+        <v>335</v>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
-        <v>327</v>
+        <v>336</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="C13" s="26">
         <v>0.2</v>
@@ -11670,15 +11739,15 @@
         <v>0</v>
       </c>
       <c r="I13" s="28" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>331</v>
+        <v>340</v>
       </c>
       <c r="C14" s="26">
         <v>0.8</v>
@@ -11691,13 +11760,13 @@
         <v>1</v>
       </c>
       <c r="I14" s="28" t="s">
-        <v>332</v>
+        <v>341</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="29"/>
       <c r="B16" s="30" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="C16" s="31">
         <f>IF(COUNT(C5:C14)&lt;10,"",(SUMSQ(C5:C14)-2*SUMPRODUCT(C5:C14,$H$5:$H$14)+SUMSQ($H$5:$H$14))/COUNT(C5:C14))</f>
@@ -11723,7 +11792,7 @@
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="29"/>
       <c r="B17" s="30" t="s">
-        <v>334</v>
+        <v>343</v>
       </c>
       <c r="C17" s="31">
         <f>IF(C16="","",IF(C16&lt;=0.25,1-C16,0))</f>
@@ -11749,7 +11818,7 @@
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="29"/>
       <c r="B18" s="30" t="s">
-        <v>335</v>
+        <v>344</v>
       </c>
       <c r="C18" s="25" t="str">
         <f>IF(C16="","",IF(C16&lt;=0.25,"Calibrado","No calibrado"))</f>
@@ -11775,7 +11844,7 @@
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="29"/>
       <c r="B20" s="2" t="s">
-        <v>336</v>
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -11805,12 +11874,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>337</v>
+        <v>346</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -12115,7 +12184,7 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
-        <v>339</v>
+        <v>348</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -12123,10 +12192,10 @@
         <v>96</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>340</v>
+        <v>349</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>341</v>
+        <v>350</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -12196,7 +12265,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="30" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="B27" s="29">
         <f>SUM(B22:B26)</f>

</xml_diff>

<commit_message>
Caso de estudio en la UTI, estilo argumentativo y nombre de la tutora
- Tutora: María Cristina Jiménez Hernández.
- Caso de estudio: proceso de admisión y matrícula de la UTI (sede Quito)
  con datos reales por levantar; datos institucionales marcados como
  pendientes. Se elimina el caso simulado IES-S.
- Capítulos 1-3 en formato de ensayo argumentativo (tesis, conclusiones
  por sección y respuesta a objeciones).
- Matriz preliminar de la UTI con 13 escenarios candidatos; referencia a
  la Ley de creación de la UTI.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/matriz/Plantilla_Matriz_Riesgos_LOPDP.xlsx
+++ b/matriz/Plantilla_Matriz_Riesgos_LOPDP.xlsx
@@ -82,13 +82,13 @@
     <t>Ejemplo</t>
   </si>
   <si>
-    <t>La fila 5 de Matriz, la fila 5 de Delphi y la columna E01 de Brier contienen valores ficticios del caso simulado IES-S. Borrarlos antes de usar la plantilla.</t>
+    <t>La fila 5 de Matriz, la fila 5 de Delphi y la columna E01 de Brier contienen valores ficticios de ejemplo. Borrarlos antes de usar la plantilla.</t>
   </si>
   <si>
     <t>Matriz de riesgos del tratamiento de datos personales — LOPDP</t>
   </si>
   <si>
-    <t>Leyenda: celdas amarillas = ingresar datos; celdas grises = fórmula (no editar). Una fila por escenario y dimensión. La fila 5 es un EJEMPLO ficticio (caso simulado IES-S): reemplazar o borrar.</t>
+    <t>Leyenda: celdas amarillas = ingresar datos; celdas grises = fórmula (no editar). Una fila por escenario y dimensión. La fila 5 es un EJEMPLO ficticio: reemplazar o borrar.</t>
   </si>
   <si>
     <t>Identificación del tratamiento</t>

</xml_diff>